<commit_message>
Them Bao Minh - Dai Thang
</commit_message>
<xml_diff>
--- a/Data_HDDT.xlsx
+++ b/Data_HDDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_render\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F435960B-7E00-4453-8515-A3F5D495F5BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9588CC02-D147-4897-A7EE-192F9135ECC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="459">
   <si>
     <t>Mã kho</t>
   </si>
@@ -1372,6 +1372,48 @@
   </si>
   <si>
     <t>KDNL068</t>
+  </si>
+  <si>
+    <t>Bảo Minh</t>
+  </si>
+  <si>
+    <t>Đại Thắng</t>
+  </si>
+  <si>
+    <t>HH051-052</t>
+  </si>
+  <si>
+    <t>HH009-012</t>
+  </si>
+  <si>
+    <t>HH050-048</t>
+  </si>
+  <si>
+    <t>HH0647</t>
+  </si>
+  <si>
+    <t>KDNL087</t>
+  </si>
+  <si>
+    <t>KDNL187</t>
+  </si>
+  <si>
+    <t>1K26TBM</t>
+  </si>
+  <si>
+    <t>1K26TĐT</t>
+  </si>
+  <si>
+    <t>KDNL088</t>
+  </si>
+  <si>
+    <t>KDNL188</t>
+  </si>
+  <si>
+    <t>HH051-053</t>
+  </si>
+  <si>
+    <t>HH009-013</t>
   </si>
 </sst>
 </file>
@@ -1860,7 +1902,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A2:Q55"/>
+  <dimension ref="A1:Q55"/>
   <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -1876,6 +1918,7 @@
     <col min="392" max="16384" width="8.42578125" style="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:17" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E2" s="1" t="s">
         <v>224</v>
@@ -3658,6 +3701,33 @@
       <c r="B50" s="10">
         <v>333814</v>
       </c>
+      <c r="D50" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="L50" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="M50" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N50" s="1" t="s">
+        <v>451</v>
+      </c>
     </row>
     <row r="51" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
@@ -3665,6 +3735,27 @@
       </c>
       <c r="B51" s="10">
         <v>63211</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="M51" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N51" s="1" t="s">
+        <v>455</v>
       </c>
     </row>
     <row r="52" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Cập nhật Lạc Quần
</commit_message>
<xml_diff>
--- a/Data_HDDT.xlsx
+++ b/Data_HDDT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_render\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9588CC02-D147-4897-A7EE-192F9135ECC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC37738-DDAC-42DB-8EB0-F58D78763691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nhap lieu" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="466">
   <si>
     <t>Mã kho</t>
   </si>
@@ -1414,6 +1414,27 @@
   </si>
   <si>
     <t>HH009-013</t>
+  </si>
+  <si>
+    <t>HH009-015</t>
+  </si>
+  <si>
+    <t>HH050-051</t>
+  </si>
+  <si>
+    <t>HH051-055</t>
+  </si>
+  <si>
+    <t>KDNL190</t>
+  </si>
+  <si>
+    <t>KDNL090</t>
+  </si>
+  <si>
+    <t>Lạc Quần</t>
+  </si>
+  <si>
+    <t>1K26TLQ</t>
   </si>
 </sst>
 </file>
@@ -1903,23 +1924,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Q55"/>
-  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="9.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" style="1" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" style="1" customWidth="1"/>
-    <col min="11" max="391" width="8.42578125" style="1" customWidth="1"/>
-    <col min="392" max="16384" width="8.42578125" style="1"/>
+    <col min="10" max="10" width="11.44140625" style="1" customWidth="1"/>
+    <col min="11" max="391" width="8.44140625" style="1" customWidth="1"/>
+    <col min="392" max="16384" width="8.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="9.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E2" s="1" t="s">
         <v>224</v>
       </c>
@@ -1951,14 +1972,14 @@
         <v>253</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>224</v>
       </c>
@@ -1999,7 +2020,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>225</v>
       </c>
@@ -2037,7 +2058,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>223</v>
       </c>
@@ -2075,7 +2096,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="6" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" s="6" customFormat="1" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>222</v>
       </c>
@@ -2119,7 +2140,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="1:17" s="6" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" s="6" customFormat="1" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="1"/>
       <c r="D8" s="4" t="s">
         <v>29</v>
@@ -2157,7 +2178,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:17" s="6" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" s="6" customFormat="1" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>35</v>
       </c>
@@ -2198,7 +2219,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:17" s="6" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" s="6" customFormat="1" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>223</v>
       </c>
@@ -2239,7 +2260,7 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11" spans="1:17" s="6" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" s="6" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>224</v>
       </c>
@@ -2279,7 +2300,7 @@
       </c>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:17" s="6" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" s="6" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>225</v>
       </c>
@@ -2319,7 +2340,7 @@
       </c>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:17" s="6" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" s="6" customFormat="1" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>222</v>
       </c>
@@ -2359,7 +2380,7 @@
       </c>
       <c r="Q13" s="1"/>
     </row>
-    <row r="14" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>374</v>
       </c>
@@ -2401,7 +2422,7 @@
       </c>
       <c r="P14" s="6"/>
     </row>
-    <row r="15" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D15" s="4" t="s">
         <v>63</v>
       </c>
@@ -2436,7 +2457,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="D16" s="4" t="s">
         <v>68</v>
@@ -2469,7 +2490,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D17" s="4" t="s">
         <v>72</v>
       </c>
@@ -2504,7 +2525,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D18" s="4" t="s">
         <v>77</v>
       </c>
@@ -2539,7 +2560,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D19" s="4" t="s">
         <v>81</v>
       </c>
@@ -2574,7 +2595,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D20" s="4" t="s">
         <v>86</v>
       </c>
@@ -2609,7 +2630,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D21" s="4" t="s">
         <v>92</v>
       </c>
@@ -2644,7 +2665,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>97</v>
       </c>
@@ -2685,7 +2706,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D23" s="4" t="s">
         <v>102</v>
       </c>
@@ -2720,7 +2741,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D24" s="4" t="s">
         <v>108</v>
       </c>
@@ -2755,7 +2776,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D25" s="4" t="s">
         <v>113</v>
       </c>
@@ -2790,7 +2811,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
         <v>117</v>
       </c>
@@ -2830,7 +2851,7 @@
       </c>
       <c r="P26" s="2"/>
     </row>
-    <row r="27" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="D27" s="4" t="s">
@@ -2864,7 +2885,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>126</v>
       </c>
@@ -2900,7 +2921,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>18</v>
       </c>
@@ -2941,7 +2962,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>34</v>
       </c>
@@ -2982,7 +3003,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>11</v>
       </c>
@@ -3023,7 +3044,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>219</v>
       </c>
@@ -3062,7 +3083,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>18</v>
       </c>
@@ -3100,7 +3121,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>34</v>
       </c>
@@ -3138,7 +3159,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>11</v>
       </c>
@@ -3176,7 +3197,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>220</v>
       </c>
@@ -3214,7 +3235,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>168</v>
       </c>
@@ -3253,7 +3274,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>18</v>
       </c>
@@ -3294,7 +3315,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
         <v>34</v>
       </c>
@@ -3335,7 +3356,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
         <v>11</v>
       </c>
@@ -3374,7 +3395,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
       <c r="B41" s="10"/>
       <c r="D41" s="1" t="s">
@@ -3408,7 +3429,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
         <v>181</v>
       </c>
@@ -3444,7 +3465,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>126</v>
       </c>
@@ -3480,7 +3501,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>18</v>
       </c>
@@ -3518,7 +3539,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>34</v>
       </c>
@@ -3556,7 +3577,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>11</v>
       </c>
@@ -3594,7 +3615,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>221</v>
       </c>
@@ -3624,7 +3645,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>18</v>
       </c>
@@ -3659,7 +3680,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>34</v>
       </c>
@@ -3694,7 +3715,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>11</v>
       </c>
@@ -3729,7 +3750,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>220</v>
       </c>
@@ -3758,13 +3779,37 @@
         <v>455</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>168</v>
       </c>
       <c r="B52" s="10"/>
-    </row>
-    <row r="53" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D52" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="M52" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N52" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
         <v>18</v>
       </c>
@@ -3772,7 +3817,7 @@
         <v>333111</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>34</v>
       </c>
@@ -3780,7 +3825,7 @@
         <v>333112</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>11</v>
       </c>

</xml_diff>